<commit_message>
changing sidebar and others
</commit_message>
<xml_diff>
--- a/backup_backend/uploads/The report of Fairshare.xlsx
+++ b/backup_backend/uploads/The report of Fairshare.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -637,6 +637,42 @@
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>13/06/26</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Room C</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>testing</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
this is merge from all branch
</commit_message>
<xml_diff>
--- a/backup_backend/uploads/The report of Fairshare.xlsx
+++ b/backup_backend/uploads/The report of Fairshare.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -673,6 +673,46 @@
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>29/06/26</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Room A</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ssdad</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>23424</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>eWallet</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>dasd</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
this is the progress after merge and fixing on the file startup
</commit_message>
<xml_diff>
--- a/backup_backend/uploads/The report of Fairshare.xlsx
+++ b/backup_backend/uploads/The report of Fairshare.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,7 +479,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -489,7 +489,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Paid</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -515,7 +515,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>eWallet</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -713,6 +713,42 @@
           <t>dasd</t>
         </is>
       </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>29/06/26</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Room A</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>